<commit_message>
30 octubre 2021 v1
</commit_message>
<xml_diff>
--- a/_downloads/02786d16357d8ee3671070d613abde23/Taller proyecto Café-variables aleatorias-CLASE.xlsx
+++ b/_downloads/02786d16357d8ee3671070d613abde23/Taller proyecto Café-variables aleatorias-CLASE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\ITM\ANÁLISIS DE RIESGOS\Talleres\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01B54CBF-F0E8-419B-B159-E572E8CB7FA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67B9CA14-C0CE-4F9A-9EF0-CA9C48B937AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="751" activeTab="7" xr2:uid="{8BF2D7D1-9628-41D3-832C-45D8E5A38172}"/>
   </bookViews>
@@ -503,10 +503,10 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm"/>
     <numFmt numFmtId="165" formatCode="####\-##"/>
     <numFmt numFmtId="166" formatCode="ddd\-dd\-mmm\-yy"/>
-    <numFmt numFmtId="168" formatCode="0.0000"/>
-    <numFmt numFmtId="169" formatCode="0.0%"/>
-    <numFmt numFmtId="170" formatCode="[$USD]\ #,##0.000;[Red]\-[$USD]\ #,##0.000"/>
-    <numFmt numFmtId="171" formatCode="0.000%"/>
+    <numFmt numFmtId="167" formatCode="0.0000"/>
+    <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="169" formatCode="[$USD]\ #,##0.000;[Red]\-[$USD]\ #,##0.000"/>
+    <numFmt numFmtId="170" formatCode="0.000%"/>
   </numFmts>
   <fonts count="31" x14ac:knownFonts="1">
     <font>
@@ -1193,7 +1193,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="168" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1236,21 +1236,21 @@
     <xf numFmtId="8" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="24" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="169" fontId="24" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="24" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="24" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="170" fontId="24" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="15" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -34662,8 +34662,8 @@
       <c r="A32" s="76" t="s">
         <v>59</v>
       </c>
-      <c r="B32" s="82" t="s">
-        <v>54</v>
+      <c r="B32" s="77" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
30 octubre de 2021 v2
</commit_message>
<xml_diff>
--- a/_downloads/02786d16357d8ee3671070d613abde23/Taller proyecto Café-variables aleatorias-CLASE.xlsx
+++ b/_downloads/02786d16357d8ee3671070d613abde23/Taller proyecto Café-variables aleatorias-CLASE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\ITM\ANÁLISIS DE RIESGOS\Talleres\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67B9CA14-C0CE-4F9A-9EF0-CA9C48B937AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AB48DDF-F68A-4AE3-8179-B7591F3D202B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="751" activeTab="7" xr2:uid="{8BF2D7D1-9628-41D3-832C-45D8E5A38172}"/>
   </bookViews>
@@ -74,30 +74,6 @@
       </text>
     </comment>
     <comment ref="A44" authorId="0" shapeId="0" xr:uid="{4CDD6A11-2E29-4D66-8DFE-4B629A81132F}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>MIGUEL JIMÉNEZ:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Se divide por 0,4536 para que quede en lb.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="A46" authorId="0" shapeId="0" xr:uid="{93131D04-27B1-4FCA-AB39-466630F35B5B}">
       <text>
         <r>
           <rPr>

</xml_diff>

<commit_message>
30 octubre 2021 v3
</commit_message>
<xml_diff>
--- a/_downloads/02786d16357d8ee3671070d613abde23/Taller proyecto Café-variables aleatorias-CLASE.xlsx
+++ b/_downloads/02786d16357d8ee3671070d613abde23/Taller proyecto Café-variables aleatorias-CLASE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\ITM\ANÁLISIS DE RIESGOS\Talleres\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AB48DDF-F68A-4AE3-8179-B7591F3D202B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D16A82A-4504-4D43-BD0D-C9659AA54CA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="751" activeTab="7" xr2:uid="{8BF2D7D1-9628-41D3-832C-45D8E5A38172}"/>
   </bookViews>
@@ -69,7 +69,7 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">
-El precio está por centados de dólar, pero al dividir por 1000 queda en dólar.</t>
+El precio está por centados de dólar, pero al dividir por 100 queda en dólar.</t>
         </r>
       </text>
     </comment>

</xml_diff>